<commit_message>
Renumber discount-optimization TC ids to be sequential
TC-DOP-EXM and TC-DOP-OPT used a tens-block scheme that grouped cases by
feature area (001, 002, 010, 011, 020...), leaving gaps in the id sequence.
Renumber both families contiguously from 001, preserving their existing
ascending order so every case keeps its position:

  TC-DOP-EXM  6 cases  -> 001..006
  TC-DOP-OPT 35 cases  -> 001..035

Covers spec test titles, dependencyGate() args, prose cross-references and
the TC ID column of the two workbooks. The workbooks are patched at the cell
level inside the xlsx zip so styling and layout are unchanged. The TestRail
CSVs carry no TC ids of their own and keep the same row order, so they need
no regeneration.

No functional change: playwright --list reports the same 967 tests.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testcases/discount-optimization/discount-optimization-exemption.xlsx
+++ b/testcases/discount-optimization/discount-optimization-exemption.xlsx
@@ -790,7 +790,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TC-DOP-EXM-010</t>
+          <t>TC-DOP-EXM-003</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -974,7 +974,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TC-DOP-EXM-011</t>
+          <t>TC-DOP-EXM-004</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TC-DOP-EXM-020</t>
+          <t>TC-DOP-EXM-005</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TC-DOP-EXM-021</t>
+          <t>TC-DOP-EXM-006</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>